<commit_message>
Paypal enabled for Hydroflask emea stores
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/Hydroflask_EMEA/GoldHydroEMEA_TestData.xlsx
+++ b/src/test/resources/TestData/Hydroflask_EMEA/GoldHydroEMEA_TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4176D3-7BE8-47D7-A6AF-10F44366DFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375B33FD-E3A0-4984-8544-E9478024E7A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2210" uniqueCount="704">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2215" uniqueCount="705">
   <si>
     <t>UserName</t>
   </si>
@@ -2177,6 +2177,9 @@
   </si>
   <si>
     <t>5VR72G68E2565U77E63D</t>
+  </si>
+  <si>
+    <t>Product_3QTY</t>
   </si>
 </sst>
 </file>
@@ -2730,7 +2733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AW75"/>
+  <dimension ref="A1:AW76"/>
   <sheetFormatPr defaultColWidth="56.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -3626,21 +3629,28 @@
         <v>694</v>
       </c>
     </row>
-    <row r="23" spans="1:49" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:49" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>603</v>
+        <v>704</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="AC23" s="42" t="s">
-        <v>600</v>
-      </c>
-      <c r="AD23" s="32"/>
-      <c r="AE23" s="22"/>
+        <v>538</v>
+      </c>
+      <c r="AD23" s="32" t="s">
+        <v>390</v>
+      </c>
+      <c r="AE23" s="22" t="s">
+        <v>587</v>
+      </c>
+      <c r="AF23" s="22" t="s">
+        <v>694</v>
+      </c>
     </row>
     <row r="24" spans="1:49" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -3652,233 +3662,213 @@
     </row>
     <row r="25" spans="1:49" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
-      <c r="AC25" s="42"/>
-      <c r="AD25" s="32" t="s">
-        <v>597</v>
-      </c>
+      <c r="AC25" s="42" t="s">
+        <v>600</v>
+      </c>
+      <c r="AD25" s="32"/>
       <c r="AE25" s="22"/>
     </row>
     <row r="26" spans="1:49" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="AC26" s="42"/>
       <c r="AD26" s="32" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="AE26" s="22"/>
     </row>
     <row r="27" spans="1:49" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>588</v>
+        <v>598</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="AC27" s="42"/>
-      <c r="AD27" s="32"/>
-      <c r="AE27" s="22" t="s">
-        <v>589</v>
-      </c>
-      <c r="AF27" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="AD27" s="32" t="s">
+        <v>599</v>
+      </c>
+      <c r="AE27" s="22"/>
+    </row>
+    <row r="28" spans="1:49" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>440</v>
+        <v>588</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="AC28" t="s">
-        <v>177</v>
-      </c>
-      <c r="AD28" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="AE28" t="s">
-        <v>177</v>
+      <c r="AC28" s="42"/>
+      <c r="AD28" s="32"/>
+      <c r="AE28" s="22" t="s">
+        <v>589</v>
       </c>
       <c r="AF28" t="s">
-        <v>39</v>
+        <v>610</v>
       </c>
     </row>
     <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>176</v>
+        <v>440</v>
       </c>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="AC29" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="AD29" s="5" t="s">
         <v>120</v>
       </c>
+      <c r="AE29" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF29" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="AD30" s="5"/>
-      <c r="AF30" t="s">
-        <v>259</v>
+      <c r="AC30" t="s">
+        <v>174</v>
+      </c>
+      <c r="AD30" s="5" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>189</v>
+        <v>175</v>
       </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
-      <c r="AL31" s="12" t="s">
-        <v>442</v>
+      <c r="AD31" s="5"/>
+      <c r="AF31" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="32" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>30</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" t="s">
-        <v>34</v>
-      </c>
-      <c r="F32" t="s">
-        <v>31</v>
-      </c>
-      <c r="G32" t="s">
-        <v>35</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>32</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="H32" s="2"/>
       <c r="I32" s="2"/>
-      <c r="AD32" s="5" t="s">
-        <v>113</v>
-      </c>
       <c r="AL32" s="12" t="s">
-        <v>585</v>
+        <v>442</v>
       </c>
     </row>
     <row r="33" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>40</v>
-      </c>
-      <c r="H33" s="2"/>
+        <v>30</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" t="s">
+        <v>34</v>
+      </c>
+      <c r="F33" t="s">
+        <v>31</v>
+      </c>
+      <c r="G33" t="s">
+        <v>35</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="I33" s="2"/>
-      <c r="AH33">
-        <v>3</v>
+      <c r="AD33" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="AL33" s="12" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="34" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>43</v>
-      </c>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="G34" s="6"/>
+        <v>40</v>
+      </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
-      <c r="Z34" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA34" s="7" t="s">
-        <v>439</v>
-      </c>
-      <c r="AB34">
-        <v>123</v>
-      </c>
-      <c r="AI34" t="s">
-        <v>478</v>
-      </c>
-      <c r="AJ34" t="s">
-        <v>579</v>
+      <c r="AH34">
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>44</v>
-      </c>
-      <c r="S35" t="s">
-        <v>150</v>
-      </c>
-      <c r="T35" t="s">
-        <v>17</v>
-      </c>
-      <c r="V35" t="s">
-        <v>19</v>
-      </c>
-      <c r="W35" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="X35" s="5" t="s">
-        <v>59</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
       <c r="Z35" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AA35" s="7" t="s">
         <v>439</v>
       </c>
       <c r="AB35">
-        <v>1234</v>
+        <v>123</v>
+      </c>
+      <c r="AI35" t="s">
+        <v>478</v>
+      </c>
+      <c r="AJ35" t="s">
+        <v>579</v>
       </c>
     </row>
     <row r="36" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>46</v>
-      </c>
-      <c r="F36" t="s">
-        <v>14</v>
-      </c>
-      <c r="G36" t="s">
-        <v>14</v>
-      </c>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+        <v>44</v>
+      </c>
+      <c r="S36" t="s">
+        <v>150</v>
+      </c>
+      <c r="T36" t="s">
+        <v>17</v>
+      </c>
+      <c r="V36" t="s">
+        <v>19</v>
+      </c>
+      <c r="W36" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="X36" s="5" t="s">
+        <v>59</v>
+      </c>
       <c r="Z36" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="AA36" s="7" t="s">
         <v>439</v>
       </c>
       <c r="AB36">
-        <v>123</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="37" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>48</v>
-      </c>
-      <c r="S37" t="s">
-        <v>150</v>
-      </c>
-      <c r="T37" t="s">
-        <v>17</v>
-      </c>
-      <c r="V37" t="s">
-        <v>19</v>
-      </c>
-      <c r="W37" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="X37" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y37" s="5" t="s">
-        <v>52</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="F37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
       <c r="Z37" s="5" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="AA37" s="7" t="s">
         <v>439</v>
@@ -3886,53 +3876,53 @@
       <c r="AB37">
         <v>123</v>
       </c>
-      <c r="AK37" s="5" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="38" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>60</v>
-      </c>
-      <c r="F38" t="s">
-        <v>50</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I38" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="S38" t="s">
+        <v>150</v>
+      </c>
+      <c r="T38" t="s">
+        <v>17</v>
+      </c>
+      <c r="V38" t="s">
+        <v>19</v>
+      </c>
+      <c r="W38" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="X38" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y38" s="5" t="s">
+        <v>52</v>
+      </c>
       <c r="Z38" s="5" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="AA38" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB38" s="5">
-        <v>1</v>
+        <v>439</v>
+      </c>
+      <c r="AB38">
+        <v>123</v>
+      </c>
+      <c r="AK38" s="5" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="39" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>55</v>
-      </c>
-      <c r="S39" t="s">
-        <v>492</v>
-      </c>
-      <c r="T39" t="s">
-        <v>494</v>
-      </c>
-      <c r="U39" t="s">
-        <v>485</v>
-      </c>
-      <c r="V39" t="s">
-        <v>493</v>
-      </c>
-      <c r="W39" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="X39" s="5" t="s">
-        <v>59</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="F39" t="s">
+        <v>50</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I39" s="2"/>
       <c r="Z39" s="5" t="s">
         <v>56</v>
       </c>
@@ -3945,13 +3935,7 @@
     </row>
     <row r="40" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>61</v>
-      </c>
-      <c r="F40" t="s">
-        <v>14</v>
-      </c>
-      <c r="G40" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="S40" t="s">
         <v>492</v>
@@ -3971,112 +3955,117 @@
       <c r="X40" s="5" t="s">
         <v>59</v>
       </c>
+      <c r="Z40" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA40" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB40" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="41" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>70</v>
-      </c>
-      <c r="D41" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="W41" s="5"/>
+        <v>61</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="S41" t="s">
+        <v>492</v>
+      </c>
+      <c r="T41" t="s">
+        <v>494</v>
+      </c>
+      <c r="U41" t="s">
+        <v>485</v>
+      </c>
+      <c r="V41" t="s">
+        <v>493</v>
+      </c>
+      <c r="W41" s="5" t="s">
+        <v>495</v>
+      </c>
       <c r="X41" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>488</v>
-      </c>
-      <c r="E42" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="H42" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="I42" s="2"/>
-      <c r="S42" t="s">
-        <v>492</v>
-      </c>
-      <c r="T42" t="s">
-        <v>494</v>
-      </c>
-      <c r="U42" t="s">
-        <v>485</v>
-      </c>
-      <c r="V42" t="s">
-        <v>493</v>
-      </c>
-      <c r="W42" s="5" t="s">
-        <v>495</v>
-      </c>
+        <v>591</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="W42" s="5"/>
       <c r="X42" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>118</v>
-      </c>
-      <c r="F43" t="s">
-        <v>14</v>
-      </c>
-      <c r="G43" t="s">
-        <v>15</v>
-      </c>
-      <c r="AL43" t="s">
-        <v>434</v>
+        <v>77</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="H43" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="I43" s="2"/>
+      <c r="S43" t="s">
+        <v>492</v>
+      </c>
+      <c r="T43" t="s">
+        <v>494</v>
+      </c>
+      <c r="U43" t="s">
+        <v>485</v>
+      </c>
+      <c r="V43" t="s">
+        <v>493</v>
+      </c>
+      <c r="W43" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="X43" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>151</v>
+        <v>118</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" t="s">
+        <v>15</v>
       </c>
       <c r="AL44" t="s">
-        <v>582</v>
-      </c>
-      <c r="AM44" t="s">
-        <v>295</v>
-      </c>
-      <c r="AN44" t="s">
-        <v>313</v>
-      </c>
-      <c r="AO44" t="s">
-        <v>313</v>
+        <v>434</v>
       </c>
     </row>
     <row r="45" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>164</v>
-      </c>
-      <c r="R45" s="12"/>
-      <c r="S45" t="s">
-        <v>492</v>
-      </c>
-      <c r="T45" t="s">
-        <v>494</v>
-      </c>
-      <c r="U45" t="s">
-        <v>485</v>
-      </c>
-      <c r="V45" t="s">
-        <v>493</v>
-      </c>
-      <c r="W45" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="X45" s="5" t="s">
-        <v>59</v>
+        <v>151</v>
+      </c>
+      <c r="AL45" t="s">
+        <v>582</v>
       </c>
       <c r="AM45" t="s">
         <v>295</v>
@@ -4090,76 +4079,98 @@
     </row>
     <row r="46" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>166</v>
-      </c>
-      <c r="F46" t="s">
-        <v>167</v>
-      </c>
-      <c r="H46" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I46" s="12"/>
-      <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
-      <c r="L46" s="12"/>
-      <c r="M46" s="12"/>
-      <c r="N46" s="12"/>
-      <c r="O46" s="12"/>
-      <c r="P46" s="12"/>
-      <c r="Q46" s="12"/>
-      <c r="AC46" t="s">
-        <v>257</v>
-      </c>
-      <c r="AP46" t="s">
-        <v>186</v>
+        <v>164</v>
+      </c>
+      <c r="R46" s="12"/>
+      <c r="S46" t="s">
+        <v>492</v>
+      </c>
+      <c r="T46" t="s">
+        <v>494</v>
+      </c>
+      <c r="U46" t="s">
+        <v>485</v>
+      </c>
+      <c r="V46" t="s">
+        <v>493</v>
+      </c>
+      <c r="W46" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="X46" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AM46" t="s">
+        <v>295</v>
+      </c>
+      <c r="AN46" t="s">
+        <v>313</v>
+      </c>
+      <c r="AO46" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="47" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>184</v>
-      </c>
-      <c r="H47" s="23" t="s">
-        <v>591</v>
+        <v>166</v>
+      </c>
+      <c r="F47" t="s">
+        <v>167</v>
+      </c>
+      <c r="H47" s="12" t="s">
+        <v>28</v>
       </c>
       <c r="I47" s="12"/>
+      <c r="J47" s="12"/>
+      <c r="K47" s="12"/>
+      <c r="L47" s="12"/>
+      <c r="M47" s="12"/>
+      <c r="N47" s="12"/>
+      <c r="O47" s="12"/>
+      <c r="P47" s="12"/>
+      <c r="Q47" s="12"/>
+      <c r="AC47" t="s">
+        <v>257</v>
+      </c>
       <c r="AP47" t="s">
-        <v>279</v>
+        <v>186</v>
       </c>
     </row>
     <row r="48" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>278</v>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="H48" s="23" t="s">
+        <v>591</v>
+      </c>
+      <c r="I48" s="12"/>
       <c r="AP48" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="49" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>283</v>
-      </c>
-      <c r="F49" t="s">
-        <v>15</v>
-      </c>
-      <c r="G49" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC49" t="s">
-        <v>255</v>
-      </c>
-      <c r="AD49" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="AF49" t="s">
-        <v>39</v>
-      </c>
-      <c r="AQ49" t="s">
-        <v>83</v>
+        <v>278</v>
+      </c>
+      <c r="AP49" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="50" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>215</v>
+        <v>283</v>
+      </c>
+      <c r="F50" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC50" t="s">
+        <v>255</v>
+      </c>
+      <c r="AD50" s="5" t="s">
+        <v>120</v>
       </c>
       <c r="AF50" t="s">
         <v>39</v>
@@ -4167,56 +4178,59 @@
       <c r="AQ50" t="s">
         <v>83</v>
       </c>
-      <c r="AR50" t="s">
-        <v>216</v>
-      </c>
-      <c r="AS50" t="s">
-        <v>214</v>
-      </c>
     </row>
     <row r="51" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>209</v>
-      </c>
-      <c r="R51" s="5"/>
+        <v>215</v>
+      </c>
+      <c r="AF51" t="s">
+        <v>39</v>
+      </c>
+      <c r="AQ51" t="s">
+        <v>83</v>
+      </c>
+      <c r="AR51" t="s">
+        <v>216</v>
+      </c>
+      <c r="AS51" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="52" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>601</v>
-      </c>
-      <c r="P52" t="s">
-        <v>602</v>
+        <v>209</v>
       </c>
       <c r="R52" s="5"/>
     </row>
     <row r="53" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>338</v>
-      </c>
-      <c r="J53" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="K53" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="L53" s="5"/>
-      <c r="M53" s="5"/>
-      <c r="O53" t="s">
-        <v>340</v>
-      </c>
-      <c r="P53" s="26" t="s">
-        <v>566</v>
-      </c>
-      <c r="Q53" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="R53" t="s">
-        <v>344</v>
-      </c>
+        <v>601</v>
+      </c>
+      <c r="P53" t="s">
+        <v>602</v>
+      </c>
+      <c r="R53" s="5"/>
     </row>
     <row r="54" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>342</v>
+        <v>338</v>
+      </c>
+      <c r="J54" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="K54" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="L54" s="5"/>
+      <c r="M54" s="5"/>
+      <c r="O54" t="s">
+        <v>340</v>
+      </c>
+      <c r="P54" s="26" t="s">
+        <v>566</v>
+      </c>
+      <c r="Q54" s="5" t="s">
+        <v>354</v>
       </c>
       <c r="R54" t="s">
         <v>344</v>
@@ -4224,157 +4238,136 @@
     </row>
     <row r="55" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>345</v>
-      </c>
-      <c r="L55" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="M55" s="5" t="s">
-        <v>498</v>
-      </c>
-      <c r="N55" s="24" t="s">
-        <v>497</v>
-      </c>
-      <c r="AP55" t="s">
-        <v>350</v>
+        <v>342</v>
+      </c>
+      <c r="R55" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="56" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>347</v>
-      </c>
-      <c r="F56" t="s">
-        <v>14</v>
-      </c>
-      <c r="G56" t="s">
-        <v>348</v>
-      </c>
-      <c r="H56" s="12" t="s">
-        <v>500</v>
+        <v>345</v>
+      </c>
+      <c r="L56" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="M56" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="N56" s="24" t="s">
+        <v>497</v>
       </c>
       <c r="AP56" t="s">
-        <v>590</v>
+        <v>350</v>
       </c>
     </row>
     <row r="57" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>352</v>
-      </c>
-      <c r="P57" s="26" t="s">
-        <v>567</v>
+        <v>347</v>
+      </c>
+      <c r="F57" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" t="s">
+        <v>348</v>
+      </c>
+      <c r="H57" s="12" t="s">
+        <v>500</v>
+      </c>
+      <c r="AP57" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="58" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>569</v>
+        <v>352</v>
       </c>
       <c r="P58" s="26" t="s">
-        <v>570</v>
-      </c>
-      <c r="S58" t="s">
-        <v>492</v>
-      </c>
-      <c r="T58" t="s">
-        <v>494</v>
-      </c>
-      <c r="U58" t="s">
-        <v>485</v>
-      </c>
-      <c r="V58" t="s">
-        <v>493</v>
-      </c>
-      <c r="W58" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="X58" s="5" t="s">
-        <v>59</v>
+        <v>567</v>
       </c>
     </row>
     <row r="59" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>201</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="D59" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F59" t="s">
-        <v>14</v>
-      </c>
-      <c r="G59" t="s">
-        <v>348</v>
-      </c>
-      <c r="H59" s="12" t="s">
-        <v>304</v>
+        <v>569</v>
+      </c>
+      <c r="P59" s="26" t="s">
+        <v>570</v>
+      </c>
+      <c r="S59" t="s">
+        <v>492</v>
+      </c>
+      <c r="T59" t="s">
+        <v>494</v>
+      </c>
+      <c r="U59" t="s">
+        <v>485</v>
+      </c>
+      <c r="V59" t="s">
+        <v>493</v>
+      </c>
+      <c r="W59" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="X59" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="60" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>362</v>
-      </c>
-      <c r="P60" s="26" t="s">
-        <v>565</v>
+        <v>201</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60" t="s">
+        <v>348</v>
+      </c>
+      <c r="H60" s="12" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="61" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>430</v>
-      </c>
-      <c r="P61" s="27" t="s">
-        <v>696</v>
+        <v>362</v>
+      </c>
+      <c r="P61" s="26" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="62" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>431</v>
-      </c>
-      <c r="P62" s="26" t="s">
-        <v>699</v>
-      </c>
-      <c r="AU62" t="s">
-        <v>513</v>
-      </c>
-      <c r="AV62" s="31" t="s">
-        <v>232</v>
+        <v>430</v>
+      </c>
+      <c r="P62" s="27" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="63" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>431</v>
+      </c>
+      <c r="P63" s="26" t="s">
+        <v>699</v>
+      </c>
+      <c r="AU63" t="s">
+        <v>513</v>
+      </c>
+      <c r="AV63" s="31" t="s">
         <v>232</v>
-      </c>
-      <c r="R63" s="33"/>
-      <c r="S63" s="33"/>
-      <c r="T63" s="33"/>
-      <c r="U63" s="33"/>
-      <c r="V63" s="33"/>
-      <c r="W63" s="33"/>
-      <c r="X63" s="33"/>
-      <c r="Y63" s="33"/>
-      <c r="Z63" s="33"/>
-      <c r="AA63" s="33"/>
-      <c r="AB63" s="33"/>
-      <c r="AC63" s="33" t="s">
-        <v>256</v>
-      </c>
-      <c r="AD63" s="33">
-        <v>1</v>
-      </c>
-      <c r="AE63" s="33"/>
-      <c r="AU63" t="s">
-        <v>692</v>
-      </c>
-      <c r="AV63" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="64" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>634</v>
+        <v>232</v>
       </c>
       <c r="R64" s="33"/>
       <c r="S64" s="33"/>
@@ -4387,11 +4380,15 @@
       <c r="Z64" s="33"/>
       <c r="AA64" s="33"/>
       <c r="AB64" s="33"/>
-      <c r="AC64" s="33"/>
-      <c r="AD64" s="33"/>
+      <c r="AC64" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="AD64" s="33">
+        <v>1</v>
+      </c>
       <c r="AE64" s="33"/>
       <c r="AU64" t="s">
-        <v>635</v>
+        <v>692</v>
       </c>
       <c r="AV64" t="s">
         <v>315</v>
@@ -4399,7 +4396,7 @@
     </row>
     <row r="65" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="R65" s="33"/>
       <c r="S65" s="33"/>
@@ -4416,15 +4413,15 @@
       <c r="AD65" s="33"/>
       <c r="AE65" s="33"/>
       <c r="AU65" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="AV65" t="s">
-        <v>638</v>
+        <v>315</v>
       </c>
     </row>
     <row r="66" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="R66" s="33"/>
       <c r="S66" s="33"/>
@@ -4441,132 +4438,157 @@
       <c r="AD66" s="33"/>
       <c r="AE66" s="33"/>
       <c r="AU66" t="s">
+        <v>639</v>
+      </c>
+      <c r="AV66" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="67" spans="1:48" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>640</v>
+      </c>
+      <c r="R67" s="33"/>
+      <c r="S67" s="33"/>
+      <c r="T67" s="33"/>
+      <c r="U67" s="33"/>
+      <c r="V67" s="33"/>
+      <c r="W67" s="33"/>
+      <c r="X67" s="33"/>
+      <c r="Y67" s="33"/>
+      <c r="Z67" s="33"/>
+      <c r="AA67" s="33"/>
+      <c r="AB67" s="33"/>
+      <c r="AC67" s="33"/>
+      <c r="AD67" s="33"/>
+      <c r="AE67" s="33"/>
+      <c r="AU67" t="s">
         <v>642</v>
       </c>
-      <c r="AV66" t="s">
+      <c r="AV67" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="67" spans="1:48" x14ac:dyDescent="0.25">
-      <c r="A67" s="33" t="s">
+    <row r="68" spans="1:48" x14ac:dyDescent="0.25">
+      <c r="A68" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="B67" s="33"/>
-      <c r="C67" s="33"/>
-      <c r="D67" s="33"/>
-      <c r="E67" s="33"/>
-      <c r="F67" s="33"/>
-      <c r="G67" s="33"/>
-      <c r="H67" s="33"/>
-      <c r="I67" s="33"/>
-      <c r="J67" s="33"/>
-      <c r="K67" s="33"/>
-      <c r="L67" s="33"/>
-      <c r="M67" s="33"/>
-      <c r="N67" s="33"/>
-      <c r="O67" s="33"/>
-      <c r="P67" s="33"/>
-      <c r="Q67" s="33"/>
-    </row>
-    <row r="68" spans="1:48" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>444</v>
-      </c>
-      <c r="P68" s="26" t="s">
-        <v>697</v>
-      </c>
+      <c r="B68" s="33"/>
+      <c r="C68" s="33"/>
+      <c r="D68" s="33"/>
+      <c r="E68" s="33"/>
+      <c r="F68" s="33"/>
+      <c r="G68" s="33"/>
+      <c r="H68" s="33"/>
+      <c r="I68" s="33"/>
+      <c r="J68" s="33"/>
+      <c r="K68" s="33"/>
+      <c r="L68" s="33"/>
+      <c r="M68" s="33"/>
+      <c r="N68" s="33"/>
+      <c r="O68" s="33"/>
+      <c r="P68" s="33"/>
+      <c r="Q68" s="33"/>
     </row>
     <row r="69" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>444</v>
+      </c>
+      <c r="P69" s="26" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="70" spans="1:48" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>499</v>
       </c>
-      <c r="P69" s="26" t="s">
+      <c r="P70" s="26" t="s">
         <v>568</v>
       </c>
-      <c r="S69" t="s">
+      <c r="S70" t="s">
         <v>509</v>
       </c>
-    </row>
-    <row r="70" spans="1:48" ht="30" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>508</v>
-      </c>
-      <c r="AC70" s="42"/>
     </row>
     <row r="71" spans="1:48" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>508</v>
+      </c>
+      <c r="AC71" s="42"/>
+    </row>
+    <row r="72" spans="1:48" ht="30" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>511</v>
       </c>
-      <c r="AC71" s="42" t="s">
+      <c r="AC72" s="42" t="s">
         <v>636</v>
-      </c>
-    </row>
-    <row r="72" spans="1:48" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>515</v>
-      </c>
-      <c r="P72" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="73" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>605</v>
+        <v>515</v>
       </c>
       <c r="P73" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
     </row>
     <row r="74" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>701</v>
+        <v>605</v>
       </c>
       <c r="P74" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
     </row>
     <row r="75" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>701</v>
+      </c>
+      <c r="P75" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="76" spans="1:48" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>702</v>
       </c>
-      <c r="P75" t="s">
+      <c r="P76" t="s">
         <v>703</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H2" r:id="rId1" xr:uid="{92F09EC2-FC6F-443B-965E-DCA7B56F1753}"/>
-    <hyperlink ref="D32" r:id="rId2" display="Lotuswave@123" xr:uid="{27A376CC-4E23-4441-B806-FE9FF359794E}"/>
+    <hyperlink ref="D33" r:id="rId2" display="Lotuswave@123" xr:uid="{27A376CC-4E23-4441-B806-FE9FF359794E}"/>
     <hyperlink ref="E2" r:id="rId3" xr:uid="{5B310480-7344-4661-AB0F-D7D61F727B40}"/>
-    <hyperlink ref="H38" r:id="rId4" xr:uid="{D3AC8605-ACE0-4742-A275-CC55BA0B713E}"/>
-    <hyperlink ref="H42" r:id="rId5" xr:uid="{EBF04138-1F63-4113-A63D-68EC86409EAF}"/>
-    <hyperlink ref="AL31" r:id="rId6" xr:uid="{C3ED735C-0638-4013-B1A9-35D874D27CCD}"/>
-    <hyperlink ref="H46" r:id="rId7" xr:uid="{7B92FAF6-FC7B-4378-BAA5-F455D3557016}"/>
+    <hyperlink ref="H39" r:id="rId4" xr:uid="{D3AC8605-ACE0-4742-A275-CC55BA0B713E}"/>
+    <hyperlink ref="H43" r:id="rId5" xr:uid="{EBF04138-1F63-4113-A63D-68EC86409EAF}"/>
+    <hyperlink ref="AL32" r:id="rId6" xr:uid="{C3ED735C-0638-4013-B1A9-35D874D27CCD}"/>
+    <hyperlink ref="H47" r:id="rId7" xr:uid="{7B92FAF6-FC7B-4378-BAA5-F455D3557016}"/>
     <hyperlink ref="D2" r:id="rId8" xr:uid="{6D9C84C2-080E-49A8-91A9-0C4040F17B99}"/>
-    <hyperlink ref="H47" r:id="rId9" display="Hfemeanewaccount@gmail.com" xr:uid="{5EDA0D22-59C6-4E86-B1C8-F3DDADDA222C}"/>
+    <hyperlink ref="H48" r:id="rId9" display="Hfemeanewaccount@gmail.com" xr:uid="{5EDA0D22-59C6-4E86-B1C8-F3DDADDA222C}"/>
     <hyperlink ref="B2" r:id="rId10" xr:uid="{49EA4C67-65EF-4ECE-B592-DD27DDBFE9D8}"/>
     <hyperlink ref="I2" r:id="rId11" xr:uid="{41758504-FDAA-49B8-A517-3CF2E58C91CC}"/>
     <hyperlink ref="C2" r:id="rId12" xr:uid="{12FE48FE-6D5F-46FF-BB71-C2756AE73EE8}"/>
     <hyperlink ref="D3" r:id="rId13" xr:uid="{62C3648F-7D52-4B9F-ADF3-7CB24D30FA17}"/>
     <hyperlink ref="E3" r:id="rId14" xr:uid="{32229FD5-4AFA-45C3-BF60-2566B7569180}"/>
     <hyperlink ref="AC19" r:id="rId15" display="https://mcloud-na-preprod.hydroflask.com/wide-mouth-flex-cap?color=Black" xr:uid="{618667E2-3380-4A1C-B34F-ABDD50D4EE61}"/>
-    <hyperlink ref="H56" r:id="rId16" xr:uid="{7BF19D0A-861B-44DA-ABCD-EB14EC4082CF}"/>
-    <hyperlink ref="H59" r:id="rId17" xr:uid="{7332F9F7-6E5B-4009-8325-28D766EC646E}"/>
+    <hyperlink ref="H57" r:id="rId16" xr:uid="{7BF19D0A-861B-44DA-ABCD-EB14EC4082CF}"/>
+    <hyperlink ref="H60" r:id="rId17" xr:uid="{7332F9F7-6E5B-4009-8325-28D766EC646E}"/>
     <hyperlink ref="E6" r:id="rId18" xr:uid="{2C317B8E-AF32-4D4C-AE44-1F2FC9B108BE}"/>
     <hyperlink ref="D6" r:id="rId19" xr:uid="{E6081600-960B-4A22-B355-F1C4E40470AA}"/>
     <hyperlink ref="B6" r:id="rId20" xr:uid="{7D100C12-0453-4673-AC35-2EA4A2603564}"/>
     <hyperlink ref="I6" r:id="rId21" display="LotusQA.GLD.PR.HYF.AutoTest7@gmail.com" xr:uid="{4380A0E0-76DF-485C-8BEA-6C28F9B24971}"/>
     <hyperlink ref="C6" r:id="rId22" display="LotusQA.GLD.PR.HYF.AutoTest7@gmail.com" xr:uid="{8F318BE4-05CB-41C2-8BFD-E5C42814E494}"/>
     <hyperlink ref="H6" r:id="rId23" xr:uid="{407C8F4E-9B49-4856-B5B1-AADA1B530463}"/>
-    <hyperlink ref="D41" r:id="rId24" xr:uid="{CFA846D7-1044-49EA-A0C9-5358EDB0782D}"/>
+    <hyperlink ref="D42" r:id="rId24" xr:uid="{CFA846D7-1044-49EA-A0C9-5358EDB0782D}"/>
     <hyperlink ref="H4" r:id="rId25" xr:uid="{D910C898-EA43-409E-B04E-9B9BFB5A3D9D}"/>
     <hyperlink ref="E4" r:id="rId26" xr:uid="{B86A9B6C-A653-4B11-A92A-B12ECCF56B54}"/>
     <hyperlink ref="D4" r:id="rId27" xr:uid="{5357CB07-F4C9-42F8-8AA6-82DE7438DA1F}"/>
     <hyperlink ref="B4" r:id="rId28" xr:uid="{6B5AE7EC-0874-471E-8B2A-119BB6055DFF}"/>
     <hyperlink ref="I4" r:id="rId29" xr:uid="{C425EF67-01D4-42EC-8E86-0A6DFDCBD4BA}"/>
     <hyperlink ref="C4" r:id="rId30" xr:uid="{50F1E974-01BC-40BB-A015-3C5D601540DD}"/>
-    <hyperlink ref="H41" r:id="rId31" display="Hfemeanewaccount@gmail.com" xr:uid="{EDD9788C-AEBE-4F86-8A6C-8043A32B81A6}"/>
-    <hyperlink ref="I41" r:id="rId32" display="Hfemeanewaccount@gmail.com" xr:uid="{68882096-6651-4D29-9355-6F1410B100AA}"/>
+    <hyperlink ref="H42" r:id="rId31" display="Hfemeanewaccount@gmail.com" xr:uid="{EDD9788C-AEBE-4F86-8A6C-8043A32B81A6}"/>
+    <hyperlink ref="I42" r:id="rId32" display="Hfemeanewaccount@gmail.com" xr:uid="{68882096-6651-4D29-9355-6F1410B100AA}"/>
     <hyperlink ref="H8" r:id="rId33" xr:uid="{867EC1A7-B881-422A-8354-C1C7FCE40AAE}"/>
     <hyperlink ref="E8" r:id="rId34" xr:uid="{5ACEF6FA-BF68-4BBD-BE65-3578FCD63C44}"/>
     <hyperlink ref="D8" r:id="rId35" xr:uid="{3607587D-2F3E-4312-8C6F-F1EF148F7A1A}"/>
@@ -4588,9 +4610,9 @@
     <hyperlink ref="B10" r:id="rId51" xr:uid="{17E9DB6C-30D3-4F48-81EA-C35AF660B980}"/>
     <hyperlink ref="I10" r:id="rId52" xr:uid="{797DAE89-D941-4743-B597-439A5C30AAF0}"/>
     <hyperlink ref="C10" r:id="rId53" xr:uid="{34EC3537-EEF4-4D6F-923E-4AE4713BD831}"/>
-    <hyperlink ref="D59" r:id="rId54" xr:uid="{D9B3D2C8-8647-42D9-A4A0-095F61674861}"/>
+    <hyperlink ref="D60" r:id="rId54" xr:uid="{D9B3D2C8-8647-42D9-A4A0-095F61674861}"/>
     <hyperlink ref="H13" r:id="rId55" xr:uid="{E9756DE8-6826-41D1-9FFA-8650413C0FFA}"/>
-    <hyperlink ref="AL32" r:id="rId56" xr:uid="{277537F5-68B0-41F9-AB74-A5237DB228B6}"/>
+    <hyperlink ref="AL33" r:id="rId56" xr:uid="{277537F5-68B0-41F9-AB74-A5237DB228B6}"/>
     <hyperlink ref="B3" r:id="rId57" xr:uid="{150B5483-771D-49C8-8086-2BA53FC3ED08}"/>
     <hyperlink ref="H3" r:id="rId58" xr:uid="{195D6A3E-A949-43F0-8B40-48EAF4295DC3}"/>
     <hyperlink ref="C3" r:id="rId59" xr:uid="{E3D4A2D5-A63D-402B-9143-60103D9905D4}"/>

</xml_diff>